<commit_message>
[feat/ASP-2730-Eswatini-SMS-Report] Removed values with pending definition.
</commit_message>
<xml_diff>
--- a/api/templates/sz_sms_stats/en.xlsx
+++ b/api/templates/sz_sms_stats/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\sz_sms_stats\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CBED2EA-BF49-4D30-82AE-D32F7C0D6911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE6778A8-9B48-4868-B8A9-BACC060FD344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E3D95321-C7DA-440A-B60E-5C29FCA416BB}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Number of test done</t>
   </si>
@@ -46,12 +46,6 @@
     <t>Number of errors/invalids</t>
   </si>
   <si>
-    <t>Number of SMS results sent to facility</t>
-  </si>
-  <si>
-    <t>Number of SMS notifications to sent to client</t>
-  </si>
-  <si>
     <t>Average TAT (Sample Collection - Registration)</t>
   </si>
   <si>
@@ -83,9 +77,6 @@
   </si>
   <si>
     <t>Number of SMS for other topics (device issues, etc.)</t>
-  </si>
-  <si>
-    <t>Pending</t>
   </si>
 </sst>
 </file>
@@ -612,7 +603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4D2576A-CB05-4187-998F-E769F2B698BE}">
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" customWidth="1"/>
@@ -620,27 +611,27 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -683,7 +674,7 @@
     <row r="11" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="12" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B12" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
@@ -695,7 +686,7 @@
     </row>
     <row r="13" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="14" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C13" s="15"/>
       <c r="D13" s="15"/>
@@ -706,97 +697,68 @@
       <c r="I13" s="16"/>
     </row>
     <row r="14" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="15" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="11" t="s">
+    <row r="15" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="19"/>
+    </row>
+    <row r="16" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="17" spans="2:13" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="13" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="14" t="s">
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="M17" s="4"/>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B18" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="16" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="2:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="18" spans="2:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="19"/>
-    </row>
-    <row r="19" spans="2:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="20" spans="2:13" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="2" t="s">
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="6"/>
+      <c r="K18" s="6"/>
+      <c r="L18" s="6"/>
+      <c r="M18" s="7"/>
+    </row>
+    <row r="19" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
-      <c r="M20" s="4"/>
-    </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B21" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="6"/>
-      <c r="L21" s="6"/>
-      <c r="M21" s="7"/>
-    </row>
-    <row r="22" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
-      <c r="K22" s="9"/>
-      <c r="L22" s="9"/>
-      <c r="M22" s="10"/>
-    </row>
-    <row r="23" spans="2:13" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9"/>
+      <c r="L19" s="9"/>
+      <c r="M19" s="10"/>
+    </row>
+    <row r="20" spans="2:13" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>